<commit_message>
Refactor paths for evaluate_architecture_metrics.py and update metrics calculations
- Updated import paths for evaluate_architecture_metrics.py in multiple scripts to reflect new directory structure.
- Added Spearman's rho calculation to scenario_rows function in cluster_bootstrap_ci.py.
- Adjusted supplementary table targets in generate_imputed_robustness_tables.py to be per model.
- Introduced a new script generate_grouped_bars_figure.py for generating grouped bar figures for overall performance by model.
- Updated run_paper_pipeline.py to reflect changes in script locations and ensure proper execution flow.
</commit_message>
<xml_diff>
--- a/Analysis/failure_inclusive_metrics.xlsx
+++ b/Analysis/failure_inclusive_metrics.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O49"/>
+  <dimension ref="A1:R49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,30 +464,45 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>spearman_rho_conditional</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>spearman_rho_inclusive</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>spearman_rho_delta</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>top1_accuracy_conditional</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>top1_accuracy_inclusive</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>top1_accuracy_delta</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>top2_accuracy_conditional</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>top2_accuracy_inclusive</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>top2_accuracy_delta</t>
         </is>
@@ -528,21 +543,30 @@
         <v>-0.0005999999999999999</v>
       </c>
       <c r="J2" t="n">
+        <v>0.0052</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.0046</v>
+      </c>
+      <c r="L2" t="n">
+        <v>-0.0005</v>
+      </c>
+      <c r="M2" t="n">
         <v>0.3171</v>
       </c>
-      <c r="K2" t="n">
+      <c r="N2" t="n">
         <v>0.3169</v>
       </c>
-      <c r="L2" t="n">
+      <c r="O2" t="n">
         <v>-0.0001</v>
       </c>
-      <c r="M2" t="n">
+      <c r="P2" t="n">
         <v>0.6308</v>
       </c>
-      <c r="N2" t="n">
+      <c r="Q2" t="n">
         <v>0.6308</v>
       </c>
-      <c r="O2" t="n">
+      <c r="R2" t="n">
         <v>-0</v>
       </c>
     </row>
@@ -581,21 +605,30 @@
         <v>0.0002</v>
       </c>
       <c r="J3" t="n">
+        <v>-0.103</v>
+      </c>
+      <c r="K3" t="n">
+        <v>-0.1029</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="M3" t="n">
         <v>0.1978</v>
       </c>
-      <c r="K3" t="n">
+      <c r="N3" t="n">
         <v>0.1981</v>
       </c>
-      <c r="L3" t="n">
+      <c r="O3" t="n">
         <v>0.0002</v>
       </c>
-      <c r="M3" t="n">
+      <c r="P3" t="n">
         <v>0.639</v>
       </c>
-      <c r="N3" t="n">
+      <c r="Q3" t="n">
         <v>0.639</v>
       </c>
-      <c r="O3" t="n">
+      <c r="R3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -634,21 +667,30 @@
         <v>-0.0011</v>
       </c>
       <c r="J4" t="n">
+        <v>0.1452</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.1441</v>
+      </c>
+      <c r="L4" t="n">
+        <v>-0.0011</v>
+      </c>
+      <c r="M4" t="n">
         <v>0.3668</v>
       </c>
-      <c r="K4" t="n">
+      <c r="N4" t="n">
         <v>0.3665</v>
       </c>
-      <c r="L4" t="n">
+      <c r="O4" t="n">
         <v>-0.0003</v>
       </c>
-      <c r="M4" t="n">
+      <c r="P4" t="n">
         <v>0.7221</v>
       </c>
-      <c r="N4" t="n">
+      <c r="Q4" t="n">
         <v>0.7217</v>
       </c>
-      <c r="O4" t="n">
+      <c r="R4" t="n">
         <v>-0.0004</v>
       </c>
     </row>
@@ -687,21 +729,30 @@
         <v>-0.0054</v>
       </c>
       <c r="J5" t="n">
+        <v>0.5891</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.5833</v>
+      </c>
+      <c r="L5" t="n">
+        <v>-0.0057</v>
+      </c>
+      <c r="M5" t="n">
         <v>0.6194</v>
       </c>
-      <c r="K5" t="n">
+      <c r="N5" t="n">
         <v>0.6167</v>
       </c>
-      <c r="L5" t="n">
+      <c r="O5" t="n">
         <v>-0.0028</v>
       </c>
-      <c r="M5" t="n">
+      <c r="P5" t="n">
         <v>0.9192</v>
       </c>
-      <c r="N5" t="n">
+      <c r="Q5" t="n">
         <v>0.9167</v>
       </c>
-      <c r="O5" t="n">
+      <c r="R5" t="n">
         <v>-0.0025</v>
       </c>
     </row>
@@ -740,21 +791,30 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
+        <v>-0.07539999999999999</v>
+      </c>
+      <c r="K6" t="n">
+        <v>-0.07539999999999999</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
         <v>0.2492</v>
       </c>
-      <c r="K6" t="n">
+      <c r="N6" t="n">
         <v>0.2492</v>
       </c>
-      <c r="L6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" t="n">
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
         <v>0.5754</v>
       </c>
-      <c r="N6" t="n">
+      <c r="Q6" t="n">
         <v>0.5754</v>
       </c>
-      <c r="O6" t="n">
+      <c r="R6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -793,21 +853,30 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
+        <v>-0.0371</v>
+      </c>
+      <c r="K7" t="n">
+        <v>-0.0371</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
         <v>0.2543</v>
       </c>
-      <c r="K7" t="n">
+      <c r="N7" t="n">
         <v>0.2543</v>
       </c>
-      <c r="L7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" t="n">
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" t="n">
         <v>0.6143</v>
       </c>
-      <c r="N7" t="n">
+      <c r="Q7" t="n">
         <v>0.6143</v>
       </c>
-      <c r="O7" t="n">
+      <c r="R7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -846,21 +915,30 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
+        <v>0.1733</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.1733</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
         <v>0.3621</v>
       </c>
-      <c r="K8" t="n">
+      <c r="N8" t="n">
         <v>0.3621</v>
       </c>
-      <c r="L8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" t="n">
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" t="n">
         <v>0.6974</v>
       </c>
-      <c r="N8" t="n">
+      <c r="Q8" t="n">
         <v>0.6974</v>
       </c>
-      <c r="O8" t="n">
+      <c r="R8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -899,21 +977,30 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
+        <v>0.6883</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.6883</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
         <v>0.61</v>
       </c>
-      <c r="K9" t="n">
+      <c r="N9" t="n">
         <v>0.61</v>
       </c>
-      <c r="L9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" t="n">
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="n">
         <v>0.9267</v>
       </c>
-      <c r="N9" t="n">
+      <c r="Q9" t="n">
         <v>0.9267</v>
       </c>
-      <c r="O9" t="n">
+      <c r="R9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -952,21 +1039,30 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
+        <v>-0.1662</v>
+      </c>
+      <c r="K10" t="n">
+        <v>-0.1662</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
         <v>0.2677</v>
       </c>
-      <c r="K10" t="n">
+      <c r="N10" t="n">
         <v>0.2677</v>
       </c>
-      <c r="L10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" t="n">
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
         <v>0.5569</v>
       </c>
-      <c r="N10" t="n">
+      <c r="Q10" t="n">
         <v>0.5569</v>
       </c>
-      <c r="O10" t="n">
+      <c r="R10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1005,21 +1101,30 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
+        <v>0.1429</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.1429</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
         <v>0.3971</v>
       </c>
-      <c r="K11" t="n">
+      <c r="N11" t="n">
         <v>0.3971</v>
       </c>
-      <c r="L11" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" t="n">
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="n">
         <v>0.7571</v>
       </c>
-      <c r="N11" t="n">
+      <c r="Q11" t="n">
         <v>0.7571</v>
       </c>
-      <c r="O11" t="n">
+      <c r="R11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1058,21 +1163,30 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
+        <v>0.0385</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.0385</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
         <v>0.3333</v>
       </c>
-      <c r="K12" t="n">
+      <c r="N12" t="n">
         <v>0.3333</v>
       </c>
-      <c r="L12" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" t="n">
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="n">
         <v>0.6646</v>
       </c>
-      <c r="N12" t="n">
+      <c r="Q12" t="n">
         <v>0.6646</v>
       </c>
-      <c r="O12" t="n">
+      <c r="R12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1111,21 +1225,30 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
+        <v>0.1383</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.1383</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
         <v>0.33</v>
       </c>
-      <c r="K13" t="n">
+      <c r="N13" t="n">
         <v>0.33</v>
       </c>
-      <c r="L13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" t="n">
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="n">
         <v>0.6733</v>
       </c>
-      <c r="N13" t="n">
+      <c r="Q13" t="n">
         <v>0.6733</v>
       </c>
-      <c r="O13" t="n">
+      <c r="R13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1164,21 +1287,30 @@
         <v>0.0001</v>
       </c>
       <c r="J14" t="n">
+        <v>-0.037</v>
+      </c>
+      <c r="K14" t="n">
+        <v>-0.0369</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="M14" t="n">
         <v>0.2315</v>
       </c>
-      <c r="K14" t="n">
+      <c r="N14" t="n">
         <v>0.2318</v>
       </c>
-      <c r="L14" t="n">
+      <c r="O14" t="n">
         <v>0.0003</v>
       </c>
-      <c r="M14" t="n">
+      <c r="P14" t="n">
         <v>0.6758999999999999</v>
       </c>
-      <c r="N14" t="n">
+      <c r="Q14" t="n">
         <v>0.6758999999999999</v>
       </c>
-      <c r="O14" t="n">
+      <c r="R14" t="n">
         <v>-0</v>
       </c>
     </row>
@@ -1217,21 +1349,30 @@
         <v>-0.0001</v>
       </c>
       <c r="J15" t="n">
+        <v>-0.0128</v>
+      </c>
+      <c r="K15" t="n">
+        <v>-0.0129</v>
+      </c>
+      <c r="L15" t="n">
+        <v>-0.0001</v>
+      </c>
+      <c r="M15" t="n">
         <v>0.3265</v>
       </c>
-      <c r="K15" t="n">
+      <c r="N15" t="n">
         <v>0.3267</v>
       </c>
-      <c r="L15" t="n">
+      <c r="O15" t="n">
         <v>0.0001</v>
       </c>
-      <c r="M15" t="n">
+      <c r="P15" t="n">
         <v>0.6735</v>
       </c>
-      <c r="N15" t="n">
+      <c r="Q15" t="n">
         <v>0.6733</v>
       </c>
-      <c r="O15" t="n">
+      <c r="R15" t="n">
         <v>-0.0001</v>
       </c>
     </row>
@@ -1270,21 +1411,30 @@
         <v>-0.0001</v>
       </c>
       <c r="J16" t="n">
+        <v>0.0078</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.0077</v>
+      </c>
+      <c r="L16" t="n">
+        <v>-0.0001</v>
+      </c>
+      <c r="M16" t="n">
         <v>0.3001</v>
       </c>
-      <c r="K16" t="n">
+      <c r="N16" t="n">
         <v>0.3002</v>
       </c>
-      <c r="L16" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" t="n">
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="n">
         <v>0.6773</v>
       </c>
-      <c r="N16" t="n">
+      <c r="Q16" t="n">
         <v>0.6773</v>
       </c>
-      <c r="O16" t="n">
+      <c r="R16" t="n">
         <v>-0</v>
       </c>
     </row>
@@ -1323,21 +1473,30 @@
         <v>0</v>
       </c>
       <c r="J17" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="n">
         <v>0.3433</v>
       </c>
-      <c r="K17" t="n">
+      <c r="N17" t="n">
         <v>0.3433</v>
       </c>
-      <c r="L17" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" t="n">
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="n">
         <v>0.6833</v>
       </c>
-      <c r="N17" t="n">
+      <c r="Q17" t="n">
         <v>0.6833</v>
       </c>
-      <c r="O17" t="n">
+      <c r="R17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1376,21 +1535,30 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
+        <v>0.4662</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0.4662</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" t="n">
         <v>0.7015</v>
       </c>
-      <c r="K18" t="n">
+      <c r="N18" t="n">
         <v>0.7015</v>
       </c>
-      <c r="L18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" t="n">
+      <c r="O18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" t="n">
         <v>0.9015</v>
       </c>
-      <c r="N18" t="n">
+      <c r="Q18" t="n">
         <v>0.9015</v>
       </c>
-      <c r="O18" t="n">
+      <c r="R18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1429,21 +1597,30 @@
         <v>0</v>
       </c>
       <c r="J19" t="n">
+        <v>0.0371</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.0371</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" t="n">
         <v>0.3286</v>
       </c>
-      <c r="K19" t="n">
+      <c r="N19" t="n">
         <v>0.3286</v>
       </c>
-      <c r="L19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" t="n">
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="n">
         <v>0.6629</v>
       </c>
-      <c r="N19" t="n">
+      <c r="Q19" t="n">
         <v>0.6629</v>
       </c>
-      <c r="O19" t="n">
+      <c r="R19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1482,21 +1659,30 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
+        <v>0.3308</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0.3308</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" t="n">
         <v>0.5354</v>
       </c>
-      <c r="K20" t="n">
+      <c r="N20" t="n">
         <v>0.5354</v>
       </c>
-      <c r="L20" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" t="n">
+      <c r="O20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" t="n">
         <v>0.8113</v>
       </c>
-      <c r="N20" t="n">
+      <c r="Q20" t="n">
         <v>0.8113</v>
       </c>
-      <c r="O20" t="n">
+      <c r="R20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1535,21 +1721,30 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
+        <v>0.5266999999999999</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0.5266999999999999</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" t="n">
         <v>0.5967</v>
       </c>
-      <c r="K21" t="n">
+      <c r="N21" t="n">
         <v>0.5967</v>
       </c>
-      <c r="L21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M21" t="n">
+      <c r="O21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" t="n">
         <v>0.8867</v>
       </c>
-      <c r="N21" t="n">
+      <c r="Q21" t="n">
         <v>0.8867</v>
       </c>
-      <c r="O21" t="n">
+      <c r="R21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1588,21 +1783,30 @@
         <v>-0.0077</v>
       </c>
       <c r="J22" t="n">
+        <v>0.3352</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0.3277</v>
+      </c>
+      <c r="L22" t="n">
+        <v>-0.0075</v>
+      </c>
+      <c r="M22" t="n">
         <v>0.5629999999999999</v>
       </c>
-      <c r="K22" t="n">
+      <c r="N22" t="n">
         <v>0.5579</v>
       </c>
-      <c r="L22" t="n">
+      <c r="O22" t="n">
         <v>-0.0051</v>
       </c>
-      <c r="M22" t="n">
+      <c r="P22" t="n">
         <v>0.7611</v>
       </c>
-      <c r="N22" t="n">
+      <c r="Q22" t="n">
         <v>0.759</v>
       </c>
-      <c r="O22" t="n">
+      <c r="R22" t="n">
         <v>-0.0021</v>
       </c>
     </row>
@@ -1641,21 +1845,30 @@
         <v>0.001</v>
       </c>
       <c r="J23" t="n">
+        <v>-0.0936</v>
+      </c>
+      <c r="K23" t="n">
+        <v>-0.0929</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0.0008</v>
+      </c>
+      <c r="M23" t="n">
         <v>0.1528</v>
       </c>
-      <c r="K23" t="n">
+      <c r="N23" t="n">
         <v>0.1543</v>
       </c>
-      <c r="L23" t="n">
+      <c r="O23" t="n">
         <v>0.0014</v>
       </c>
-      <c r="M23" t="n">
+      <c r="P23" t="n">
         <v>0.6657</v>
       </c>
-      <c r="N23" t="n">
+      <c r="Q23" t="n">
         <v>0.6657</v>
       </c>
-      <c r="O23" t="n">
+      <c r="R23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1694,21 +1907,30 @@
         <v>-0.0032</v>
       </c>
       <c r="J24" t="n">
+        <v>0.328</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0.3246</v>
+      </c>
+      <c r="L24" t="n">
+        <v>-0.0034</v>
+      </c>
+      <c r="M24" t="n">
         <v>0.4871</v>
       </c>
-      <c r="K24" t="n">
+      <c r="N24" t="n">
         <v>0.4855</v>
       </c>
-      <c r="L24" t="n">
+      <c r="O24" t="n">
         <v>-0.0016</v>
       </c>
-      <c r="M24" t="n">
+      <c r="P24" t="n">
         <v>0.7958</v>
       </c>
-      <c r="N24" t="n">
+      <c r="Q24" t="n">
         <v>0.7945</v>
       </c>
-      <c r="O24" t="n">
+      <c r="R24" t="n">
         <v>-0.0013</v>
       </c>
     </row>
@@ -1747,21 +1969,30 @@
         <v>0</v>
       </c>
       <c r="J25" t="n">
+        <v>0.8083</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0.8083</v>
+      </c>
+      <c r="L25" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" t="n">
         <v>0.7933</v>
       </c>
-      <c r="K25" t="n">
+      <c r="N25" t="n">
         <v>0.7933</v>
       </c>
-      <c r="L25" t="n">
-        <v>0</v>
-      </c>
-      <c r="M25" t="n">
+      <c r="O25" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" t="n">
         <v>0.9833</v>
       </c>
-      <c r="N25" t="n">
+      <c r="Q25" t="n">
         <v>0.9833</v>
       </c>
-      <c r="O25" t="n">
+      <c r="R25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1800,21 +2031,30 @@
         <v>0</v>
       </c>
       <c r="J26" t="n">
+        <v>-0.0769</v>
+      </c>
+      <c r="K26" t="n">
+        <v>-0.0769</v>
+      </c>
+      <c r="L26" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" t="n">
         <v>0.3046</v>
       </c>
-      <c r="K26" t="n">
+      <c r="N26" t="n">
         <v>0.3046</v>
       </c>
-      <c r="L26" t="n">
-        <v>0</v>
-      </c>
-      <c r="M26" t="n">
+      <c r="O26" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" t="n">
         <v>0.5938</v>
       </c>
-      <c r="N26" t="n">
+      <c r="Q26" t="n">
         <v>0.5938</v>
       </c>
-      <c r="O26" t="n">
+      <c r="R26" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1853,21 +2093,30 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
+        <v>0.3014</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0.3014</v>
+      </c>
+      <c r="L27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" t="n">
         <v>0.4686</v>
       </c>
-      <c r="K27" t="n">
+      <c r="N27" t="n">
         <v>0.4686</v>
       </c>
-      <c r="L27" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" t="n">
+      <c r="O27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" t="n">
         <v>0.7743</v>
       </c>
-      <c r="N27" t="n">
+      <c r="Q27" t="n">
         <v>0.7743</v>
       </c>
-      <c r="O27" t="n">
+      <c r="R27" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1906,21 +2155,30 @@
         <v>0</v>
       </c>
       <c r="J28" t="n">
+        <v>0.2908</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0.2908</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" t="n">
         <v>0.4738</v>
       </c>
-      <c r="K28" t="n">
+      <c r="N28" t="n">
         <v>0.4738</v>
       </c>
-      <c r="L28" t="n">
-        <v>0</v>
-      </c>
-      <c r="M28" t="n">
+      <c r="O28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" t="n">
         <v>0.7651</v>
       </c>
-      <c r="N28" t="n">
+      <c r="Q28" t="n">
         <v>0.7651</v>
       </c>
-      <c r="O28" t="n">
+      <c r="R28" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1959,21 +2217,30 @@
         <v>0</v>
       </c>
       <c r="J29" t="n">
+        <v>0.6767</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0.6767</v>
+      </c>
+      <c r="L29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" t="n">
         <v>0.6633</v>
       </c>
-      <c r="K29" t="n">
+      <c r="N29" t="n">
         <v>0.6633</v>
       </c>
-      <c r="L29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M29" t="n">
+      <c r="O29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P29" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="N29" t="n">
+      <c r="Q29" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="O29" t="n">
+      <c r="R29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2012,21 +2279,30 @@
         <v>0</v>
       </c>
       <c r="J30" t="n">
+        <v>0.2415</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0.2415</v>
+      </c>
+      <c r="L30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" t="n">
         <v>0.52</v>
       </c>
-      <c r="K30" t="n">
+      <c r="N30" t="n">
         <v>0.52</v>
       </c>
-      <c r="L30" t="n">
-        <v>0</v>
-      </c>
-      <c r="M30" t="n">
+      <c r="O30" t="n">
+        <v>0</v>
+      </c>
+      <c r="P30" t="n">
         <v>0.8092</v>
       </c>
-      <c r="N30" t="n">
+      <c r="Q30" t="n">
         <v>0.8092</v>
       </c>
-      <c r="O30" t="n">
+      <c r="R30" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2065,21 +2341,30 @@
         <v>0</v>
       </c>
       <c r="J31" t="n">
+        <v>0.1829</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0.1829</v>
+      </c>
+      <c r="L31" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" t="n">
         <v>0.4114</v>
       </c>
-      <c r="K31" t="n">
+      <c r="N31" t="n">
         <v>0.4114</v>
       </c>
-      <c r="L31" t="n">
-        <v>0</v>
-      </c>
-      <c r="M31" t="n">
+      <c r="O31" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" t="n">
         <v>0.7714</v>
       </c>
-      <c r="N31" t="n">
+      <c r="Q31" t="n">
         <v>0.7714</v>
       </c>
-      <c r="O31" t="n">
+      <c r="R31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2118,21 +2403,30 @@
         <v>0</v>
       </c>
       <c r="J32" t="n">
+        <v>0.2241</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0.2241</v>
+      </c>
+      <c r="L32" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" t="n">
         <v>0.4656</v>
       </c>
-      <c r="K32" t="n">
+      <c r="N32" t="n">
         <v>0.4656</v>
       </c>
-      <c r="L32" t="n">
-        <v>0</v>
-      </c>
-      <c r="M32" t="n">
+      <c r="O32" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" t="n">
         <v>0.7805</v>
       </c>
-      <c r="N32" t="n">
+      <c r="Q32" t="n">
         <v>0.7805</v>
       </c>
-      <c r="O32" t="n">
+      <c r="R32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2171,21 +2465,30 @@
         <v>0</v>
       </c>
       <c r="J33" t="n">
+        <v>0.2533</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0.2533</v>
+      </c>
+      <c r="L33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" t="n">
         <v>0.47</v>
       </c>
-      <c r="K33" t="n">
+      <c r="N33" t="n">
         <v>0.47</v>
       </c>
-      <c r="L33" t="n">
-        <v>0</v>
-      </c>
-      <c r="M33" t="n">
+      <c r="O33" t="n">
+        <v>0</v>
+      </c>
+      <c r="P33" t="n">
         <v>0.76</v>
       </c>
-      <c r="N33" t="n">
+      <c r="Q33" t="n">
         <v>0.76</v>
       </c>
-      <c r="O33" t="n">
+      <c r="R33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2224,21 +2527,30 @@
         <v>0</v>
       </c>
       <c r="J34" t="n">
+        <v>0.9815</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0.9815</v>
+      </c>
+      <c r="L34" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" t="n">
         <v>0.9846</v>
       </c>
-      <c r="K34" t="n">
+      <c r="N34" t="n">
         <v>0.9846</v>
       </c>
-      <c r="L34" t="n">
-        <v>0</v>
-      </c>
-      <c r="M34" t="n">
+      <c r="O34" t="n">
+        <v>0</v>
+      </c>
+      <c r="P34" t="n">
         <v>1</v>
       </c>
-      <c r="N34" t="n">
+      <c r="Q34" t="n">
         <v>1</v>
       </c>
-      <c r="O34" t="n">
+      <c r="R34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2277,21 +2589,30 @@
         <v>-0.0026</v>
       </c>
       <c r="J35" t="n">
+        <v>0.9327</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="L35" t="n">
+        <v>-0.0027</v>
+      </c>
+      <c r="M35" t="n">
         <v>0.9198</v>
       </c>
-      <c r="K35" t="n">
+      <c r="N35" t="n">
         <v>0.9181</v>
       </c>
-      <c r="L35" t="n">
+      <c r="O35" t="n">
         <v>-0.0017</v>
       </c>
-      <c r="M35" t="n">
+      <c r="P35" t="n">
         <v>0.9885</v>
       </c>
-      <c r="N35" t="n">
+      <c r="Q35" t="n">
         <v>0.9876</v>
       </c>
-      <c r="O35" t="n">
+      <c r="R35" t="n">
         <v>-0.0009</v>
       </c>
     </row>
@@ -2330,21 +2651,30 @@
         <v>-0.0009</v>
       </c>
       <c r="J36" t="n">
+        <v>0.9102</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0.9092</v>
+      </c>
+      <c r="L36" t="n">
+        <v>-0.0009</v>
+      </c>
+      <c r="M36" t="n">
         <v>0.9076</v>
       </c>
-      <c r="K36" t="n">
+      <c r="N36" t="n">
         <v>0.907</v>
       </c>
-      <c r="L36" t="n">
+      <c r="O36" t="n">
         <v>-0.0005999999999999999</v>
       </c>
-      <c r="M36" t="n">
+      <c r="P36" t="n">
         <v>0.9774</v>
       </c>
-      <c r="N36" t="n">
+      <c r="Q36" t="n">
         <v>0.9771</v>
       </c>
-      <c r="O36" t="n">
+      <c r="R36" t="n">
         <v>-0.0003</v>
       </c>
     </row>
@@ -2383,21 +2713,30 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
+        <v>0.8067</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0.8067</v>
+      </c>
+      <c r="L37" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" t="n">
         <v>0.8100000000000001</v>
       </c>
-      <c r="K37" t="n">
+      <c r="N37" t="n">
         <v>0.8100000000000001</v>
       </c>
-      <c r="L37" t="n">
-        <v>0</v>
-      </c>
-      <c r="M37" t="n">
+      <c r="O37" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="N37" t="n">
+      <c r="Q37" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="O37" t="n">
+      <c r="R37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2445,12 +2784,21 @@
         <v>0</v>
       </c>
       <c r="M38" t="n">
+        <v>0.9692</v>
+      </c>
+      <c r="N38" t="n">
+        <v>0.9692</v>
+      </c>
+      <c r="O38" t="n">
+        <v>0</v>
+      </c>
+      <c r="P38" t="n">
         <v>1</v>
       </c>
-      <c r="N38" t="n">
+      <c r="Q38" t="n">
         <v>1</v>
       </c>
-      <c r="O38" t="n">
+      <c r="R38" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2489,21 +2837,30 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
+        <v>0.9829</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0.9829</v>
+      </c>
+      <c r="L39" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" t="n">
         <v>0.9657</v>
       </c>
-      <c r="K39" t="n">
+      <c r="N39" t="n">
         <v>0.9657</v>
       </c>
-      <c r="L39" t="n">
-        <v>0</v>
-      </c>
-      <c r="M39" t="n">
+      <c r="O39" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" t="n">
         <v>1</v>
       </c>
-      <c r="N39" t="n">
+      <c r="Q39" t="n">
         <v>1</v>
       </c>
-      <c r="O39" t="n">
+      <c r="R39" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2542,21 +2899,30 @@
         <v>0</v>
       </c>
       <c r="J40" t="n">
+        <v>0.9349</v>
+      </c>
+      <c r="K40" t="n">
+        <v>0.9349</v>
+      </c>
+      <c r="L40" t="n">
+        <v>0</v>
+      </c>
+      <c r="M40" t="n">
         <v>0.9313</v>
       </c>
-      <c r="K40" t="n">
+      <c r="N40" t="n">
         <v>0.9313</v>
       </c>
-      <c r="L40" t="n">
-        <v>0</v>
-      </c>
-      <c r="M40" t="n">
+      <c r="O40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P40" t="n">
         <v>0.9846</v>
       </c>
-      <c r="N40" t="n">
+      <c r="Q40" t="n">
         <v>0.9846</v>
       </c>
-      <c r="O40" t="n">
+      <c r="R40" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2595,21 +2961,30 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
+        <v>0.8417</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0.8417</v>
+      </c>
+      <c r="L41" t="n">
+        <v>0</v>
+      </c>
+      <c r="M41" t="n">
         <v>0.85</v>
       </c>
-      <c r="K41" t="n">
+      <c r="N41" t="n">
         <v>0.85</v>
       </c>
-      <c r="L41" t="n">
-        <v>0</v>
-      </c>
-      <c r="M41" t="n">
+      <c r="O41" t="n">
+        <v>0</v>
+      </c>
+      <c r="P41" t="n">
         <v>0.95</v>
       </c>
-      <c r="N41" t="n">
+      <c r="Q41" t="n">
         <v>0.95</v>
       </c>
-      <c r="O41" t="n">
+      <c r="R41" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2648,21 +3023,30 @@
         <v>0</v>
       </c>
       <c r="J42" t="n">
+        <v>0.9754</v>
+      </c>
+      <c r="K42" t="n">
+        <v>0.9754</v>
+      </c>
+      <c r="L42" t="n">
+        <v>0</v>
+      </c>
+      <c r="M42" t="n">
         <v>0.9877</v>
       </c>
-      <c r="K42" t="n">
+      <c r="N42" t="n">
         <v>0.9877</v>
       </c>
-      <c r="L42" t="n">
-        <v>0</v>
-      </c>
-      <c r="M42" t="n">
+      <c r="O42" t="n">
+        <v>0</v>
+      </c>
+      <c r="P42" t="n">
         <v>1</v>
       </c>
-      <c r="N42" t="n">
+      <c r="Q42" t="n">
         <v>1</v>
       </c>
-      <c r="O42" t="n">
+      <c r="R42" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2701,21 +3085,30 @@
         <v>-0.3152</v>
       </c>
       <c r="J43" t="n">
+        <v>0.9571</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0.6371</v>
+      </c>
+      <c r="L43" t="n">
+        <v>-0.32</v>
+      </c>
+      <c r="M43" t="n">
         <v>0.9399</v>
       </c>
-      <c r="K43" t="n">
+      <c r="N43" t="n">
         <v>0.7371</v>
       </c>
-      <c r="L43" t="n">
+      <c r="O43" t="n">
         <v>-0.2027</v>
       </c>
-      <c r="M43" t="n">
+      <c r="P43" t="n">
         <v>1</v>
       </c>
-      <c r="N43" t="n">
+      <c r="Q43" t="n">
         <v>0.8885999999999999</v>
       </c>
-      <c r="O43" t="n">
+      <c r="R43" t="n">
         <v>-0.1114</v>
       </c>
     </row>
@@ -2754,21 +3147,30 @@
         <v>-0.1077</v>
       </c>
       <c r="J44" t="n">
+        <v>0.9114</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0.8021</v>
+      </c>
+      <c r="L44" t="n">
+        <v>-0.1093</v>
+      </c>
+      <c r="M44" t="n">
         <v>0.9173</v>
       </c>
-      <c r="K44" t="n">
+      <c r="N44" t="n">
         <v>0.8472</v>
       </c>
-      <c r="L44" t="n">
+      <c r="O44" t="n">
         <v>-0.0701</v>
       </c>
-      <c r="M44" t="n">
+      <c r="P44" t="n">
         <v>0.9813</v>
       </c>
-      <c r="N44" t="n">
+      <c r="Q44" t="n">
         <v>0.9436</v>
       </c>
-      <c r="O44" t="n">
+      <c r="R44" t="n">
         <v>-0.0377</v>
       </c>
     </row>
@@ -2807,21 +3209,30 @@
         <v>0</v>
       </c>
       <c r="J45" t="n">
+        <v>0.8067</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0.8067</v>
+      </c>
+      <c r="L45" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" t="n">
         <v>0.8233</v>
       </c>
-      <c r="K45" t="n">
+      <c r="N45" t="n">
         <v>0.8233</v>
       </c>
-      <c r="L45" t="n">
-        <v>0</v>
-      </c>
-      <c r="M45" t="n">
+      <c r="O45" t="n">
+        <v>0</v>
+      </c>
+      <c r="P45" t="n">
         <v>0.9467</v>
       </c>
-      <c r="N45" t="n">
+      <c r="Q45" t="n">
         <v>0.9467</v>
       </c>
-      <c r="O45" t="n">
+      <c r="R45" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2860,21 +3271,30 @@
         <v>0</v>
       </c>
       <c r="J46" t="n">
+        <v>0.9092</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0.9092</v>
+      </c>
+      <c r="L46" t="n">
+        <v>0</v>
+      </c>
+      <c r="M46" t="n">
         <v>0.9292</v>
       </c>
-      <c r="K46" t="n">
+      <c r="N46" t="n">
         <v>0.9292</v>
       </c>
-      <c r="L46" t="n">
-        <v>0</v>
-      </c>
-      <c r="M46" t="n">
+      <c r="O46" t="n">
+        <v>0</v>
+      </c>
+      <c r="P46" t="n">
         <v>0.9815</v>
       </c>
-      <c r="N46" t="n">
+      <c r="Q46" t="n">
         <v>0.9815</v>
       </c>
-      <c r="O46" t="n">
+      <c r="R46" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2913,21 +3333,30 @@
         <v>-0.0051</v>
       </c>
       <c r="J47" t="n">
+        <v>0.8966</v>
+      </c>
+      <c r="K47" t="n">
+        <v>0.8914</v>
+      </c>
+      <c r="L47" t="n">
+        <v>-0.0052</v>
+      </c>
+      <c r="M47" t="n">
         <v>0.8737</v>
       </c>
-      <c r="K47" t="n">
+      <c r="N47" t="n">
         <v>0.8705000000000001</v>
       </c>
-      <c r="L47" t="n">
+      <c r="O47" t="n">
         <v>-0.0032</v>
       </c>
-      <c r="M47" t="n">
+      <c r="P47" t="n">
         <v>0.9713000000000001</v>
       </c>
-      <c r="N47" t="n">
+      <c r="Q47" t="n">
         <v>0.9695</v>
       </c>
-      <c r="O47" t="n">
+      <c r="R47" t="n">
         <v>-0.0018</v>
       </c>
     </row>
@@ -2966,21 +3395,30 @@
         <v>-0.0018</v>
       </c>
       <c r="J48" t="n">
+        <v>0.8895</v>
+      </c>
+      <c r="K48" t="n">
+        <v>0.8877</v>
+      </c>
+      <c r="L48" t="n">
+        <v>-0.0018</v>
+      </c>
+      <c r="M48" t="n">
         <v>0.8972</v>
       </c>
-      <c r="K48" t="n">
+      <c r="N48" t="n">
         <v>0.8961</v>
       </c>
-      <c r="L48" t="n">
+      <c r="O48" t="n">
         <v>-0.0012</v>
       </c>
-      <c r="M48" t="n">
+      <c r="P48" t="n">
         <v>0.9692</v>
       </c>
-      <c r="N48" t="n">
+      <c r="Q48" t="n">
         <v>0.9685</v>
       </c>
-      <c r="O48" t="n">
+      <c r="R48" t="n">
         <v>-0.0005999999999999999</v>
       </c>
     </row>
@@ -3019,21 +3457,30 @@
         <v>0</v>
       </c>
       <c r="J49" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="K49" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="L49" t="n">
+        <v>0</v>
+      </c>
+      <c r="M49" t="n">
         <v>0.89</v>
       </c>
-      <c r="K49" t="n">
+      <c r="N49" t="n">
         <v>0.89</v>
       </c>
-      <c r="L49" t="n">
-        <v>0</v>
-      </c>
-      <c r="M49" t="n">
+      <c r="O49" t="n">
+        <v>0</v>
+      </c>
+      <c r="P49" t="n">
         <v>0.9533</v>
       </c>
-      <c r="N49" t="n">
+      <c r="Q49" t="n">
         <v>0.9533</v>
       </c>
-      <c r="O49" t="n">
+      <c r="R49" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>